<commit_message>
sync: envy · 2026-06-29 11:33:13
</commit_message>
<xml_diff>
--- a/fase_2/precios/lista_escolar_26_27.xlsx
+++ b/fase_2/precios/lista_escolar_26_27.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B296"/>
+  <dimension ref="A1:B386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -561,17 +561,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1325650</t>
+          <t>1315629</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>870</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1316215</t>
+          <t>1325650</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -581,17 +581,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1227638</t>
+          <t>1316215</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>830</v>
+        <v>870</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1340019</t>
+          <t>1227638</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -601,247 +601,247 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1340018</t>
+          <t>1340019</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>760</v>
+        <v>830</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1340039</t>
+          <t>1340018</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>880</v>
+        <v>760</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1340020</t>
+          <t>1340039</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>760</v>
+        <v>880</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1160347</t>
+          <t>1340020</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>740</v>
+        <v>760</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1340038</t>
+          <t>1160347</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>870</v>
+        <v>740</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1160346</t>
+          <t>1340038</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>730</v>
+        <v>870</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1344025</t>
+          <t>1315631</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>670</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>947265</t>
+          <t>1160346</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>760</v>
+        <v>730</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1316216</t>
+          <t>1344025</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>870</v>
+        <v>670</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1172417</t>
+          <t>947265</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1250</v>
+        <v>760</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1337387</t>
+          <t>1316216</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1070</v>
+        <v>870</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>179643</t>
+          <t>1172417</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>730</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1345501</t>
+          <t>1337387</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1150</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>952677</t>
+          <t>179643</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1070</v>
+        <v>730</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>825682</t>
+          <t>1345501</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1090</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>960678</t>
+          <t>952677</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1110</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1340138</t>
+          <t>825682</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1010</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1053336</t>
+          <t>960678</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1070</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1099395</t>
+          <t>1340138</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1110</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1256049</t>
+          <t>1053336</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1170</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1254896</t>
+          <t>1099395</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>920</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1340048</t>
+          <t>1256049</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>830</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1341195</t>
+          <t>1254896</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>620</v>
+        <v>920</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1341196</t>
+          <t>1340048</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>620</v>
+        <v>830</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1341197</t>
+          <t>1341195</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -851,197 +851,197 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1315630</t>
+          <t>1341196</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1150</v>
+        <v>620</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1341200</t>
+          <t>1341197</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1010</v>
+        <v>620</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1315635</t>
+          <t>1315628</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1150</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1257364</t>
+          <t>1315630</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>990</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1340050</t>
+          <t>1341200</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1070</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1340046</t>
+          <t>1315635</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>760</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1341136</t>
+          <t>1257364</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>980</v>
+        <v>990</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1172396</t>
+          <t>1340050</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>770</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1160351</t>
+          <t>1340046</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>650</v>
+        <v>760</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1160352</t>
+          <t>1341136</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>650</v>
+        <v>980</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1341138</t>
+          <t>1172396</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>980</v>
+        <v>770</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1254895</t>
+          <t>1160351</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>900</v>
+        <v>650</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1341135</t>
+          <t>1160352</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1010</v>
+        <v>650</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1340044</t>
+          <t>1341138</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>760</v>
+        <v>980</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1338645</t>
+          <t>1254895</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>760</v>
+        <v>900</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>1340045</t>
+          <t>1341135</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>760</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>1344638</t>
+          <t>1340044</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>530</v>
+        <v>760</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>1344026</t>
+          <t>1338645</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>660</v>
+        <v>760</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1342195</t>
+          <t>1340045</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1200</v>
+        <v>760</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>1341194</t>
+          <t>1344638</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1051,57 +1051,57 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1337543</t>
+          <t>1344026</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>860</v>
+        <v>660</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1340136</t>
+          <t>1342195</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1010</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>1338644</t>
+          <t>1341194</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>760</v>
+        <v>530</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1340043</t>
+          <t>1337543</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>760</v>
+        <v>860</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>1340040</t>
+          <t>1340136</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>760</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1340041</t>
+          <t>1338644</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1111,277 +1111,277 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>1342194</t>
+          <t>1340043</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>980</v>
+        <v>760</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>1341191</t>
+          <t>1340040</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>590</v>
+        <v>760</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>1254894</t>
+          <t>1340041</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>1098082</t>
+          <t>1342194</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>760</v>
+        <v>980</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>1256048</t>
+          <t>1341191</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1090</v>
+        <v>590</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>179005</t>
+          <t>1254894</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1100</v>
+        <v>900</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>1247615</t>
+          <t>1098082</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1000</v>
+        <v>760</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>1340042</t>
+          <t>1256048</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>760</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>1254863</t>
+          <t>179005</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>860</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>1099355</t>
+          <t>1247615</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>1010</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>825324</t>
+          <t>1340042</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>1180</v>
+        <v>760</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>144933</t>
+          <t>1254863</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>720</v>
+        <v>860</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>1342192</t>
+          <t>1099355</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>970</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>1342193</t>
+          <t>825324</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>520</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>1341193</t>
+          <t>144933</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>580</v>
+        <v>720</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>1342196</t>
+          <t>1342192</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>660</v>
+        <v>970</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>1343975</t>
+          <t>1342193</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>1090</v>
+        <v>520</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>1315636</t>
+          <t>1341193</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>990</v>
+        <v>580</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>1173688</t>
+          <t>1342196</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>900</v>
+        <v>660</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>1256316</t>
+          <t>1343975</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>1100</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>1343976</t>
+          <t>1315636</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>970</v>
+        <v>990</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>1342190</t>
+          <t>1173688</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>940</v>
+        <v>900</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>1175958</t>
+          <t>1256316</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>1150</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>1342191</t>
+          <t>1343976</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>940</v>
+        <v>970</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>1257440</t>
+          <t>1342190</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>1100</v>
+        <v>940</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>1340017</t>
+          <t>1175958</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1100</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>1340015</t>
+          <t>1342191</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>1100</v>
+        <v>940</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>1340016</t>
+          <t>1257440</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1391,227 +1391,227 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>1254898</t>
+          <t>1340017</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>860</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>1338652</t>
+          <t>1340015</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>860</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>1338651</t>
+          <t>1340016</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>860</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>1341192</t>
+          <t>1254898</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>530</v>
+        <v>860</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>1341190</t>
+          <t>1338652</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>1070</v>
+        <v>860</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>1344637</t>
+          <t>1338651</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>990</v>
+        <v>860</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>1338196</t>
+          <t>1341192</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>970</v>
+        <v>530</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>1098695</t>
+          <t>1341190</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>900</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>1053437</t>
+          <t>1344637</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>880</v>
+        <v>990</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>1254868</t>
+          <t>1338196</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>820</v>
+        <v>970</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>825684</t>
+          <t>1098695</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>920</v>
+        <v>900</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>1340049</t>
+          <t>1053437</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>1070</v>
+        <v>880</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>1173699</t>
+          <t>1254868</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>610</v>
+        <v>820</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>1337544</t>
+          <t>825684</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>820</v>
+        <v>920</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>947278</t>
+          <t>1340049</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>760</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>1338195</t>
+          <t>1173699</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>880</v>
+        <v>610</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>1337539</t>
+          <t>1337544</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>1180</v>
+        <v>820</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>1340131</t>
+          <t>947278</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>1130</v>
+        <v>760</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>1340092</t>
+          <t>1338195</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>920</v>
+        <v>880</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>1340654</t>
+          <t>1337539</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>1090</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>1340137</t>
+          <t>1340131</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>940</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>1173629</t>
+          <t>1340092</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>990</v>
+        <v>920</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>1340653</t>
+          <t>1340654</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -1621,527 +1621,527 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>1344111</t>
+          <t>1340137</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>1100</v>
+        <v>940</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>1255687</t>
+          <t>1173629</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>1100</v>
+        <v>990</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>1340099</t>
+          <t>1340653</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>1250</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>1344112</t>
+          <t>1344111</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>650</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>1340652</t>
+          <t>1340097</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>860</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>1255688</t>
+          <t>1173634</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>1100</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>1340093</t>
+          <t>1255687</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>920</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>1337540</t>
+          <t>1340099</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>1200</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>1337541</t>
+          <t>1344112</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>1180</v>
+        <v>650</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>1095350</t>
+          <t>1340652</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>1150</v>
+        <v>860</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>1338197</t>
+          <t>952693</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>900</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>1255691</t>
+          <t>1255688</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>980</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>1255692</t>
+          <t>952694</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>990</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>1340656</t>
+          <t>1254899</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>950</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>1315632</t>
+          <t>1247619</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>1200</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>1340135</t>
+          <t>1254900</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>860</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>1340655</t>
+          <t>1053470</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>950</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>1340133</t>
+          <t>1340098</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>860</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>1340134</t>
+          <t>1340093</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>860</v>
+        <v>920</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>1256317</t>
+          <t>1337540</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1130</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>1340126</t>
+          <t>1337541</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>1130</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>1342483</t>
+          <t>1095350</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>820</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>1338650</t>
+          <t>1338197</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>920</v>
+        <v>900</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>1340094</t>
+          <t>1254902</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>900</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>1344113</t>
+          <t>1255691</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>650</v>
+        <v>980</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>1340100</t>
+          <t>1255692</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>1200</v>
+        <v>990</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>1340121</t>
+          <t>557212</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>1100</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>1256051</t>
+          <t>1340656</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>1200</v>
+        <v>950</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>1247616</t>
+          <t>1315632</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>1150</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>179655</t>
+          <t>1340135</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>530</v>
+        <v>860</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>1098112</t>
+          <t>1340655</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>660</v>
+        <v>950</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>1337542</t>
+          <t>1340133</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>1150</v>
+        <v>860</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>1340132</t>
+          <t>1340134</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>1010</v>
+        <v>860</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>1095354</t>
+          <t>1256317</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>1150</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>1338198</t>
+          <t>1340126</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>860</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>1173630</t>
+          <t>1342483</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>940</v>
+        <v>820</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>952696</t>
+          <t>1338650</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>1150</v>
+        <v>920</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>1099340</t>
+          <t>1340094</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>820</v>
+        <v>900</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>1173613</t>
+          <t>1344113</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>1130</v>
+        <v>650</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>825327</t>
+          <t>1340100</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>1220</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>1254903</t>
+          <t>1340121</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>1210</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>1340103</t>
+          <t>1256051</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>1130</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>1338199</t>
+          <t>1247616</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>860</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>1338200</t>
+          <t>179655</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>830</v>
+        <v>530</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>1095355</t>
+          <t>1098112</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>1000</v>
+        <v>660</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>1247617</t>
+          <t>1337542</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>1000</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>1315633</t>
+          <t>1340132</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>1000</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>1340104</t>
+          <t>1095354</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>1130</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>1342229</t>
+          <t>1338198</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>700</v>
+        <v>860</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>1254880</t>
+          <t>1173630</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>860</v>
+        <v>940</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>1255867</t>
+          <t>952696</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>1070</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>1340657</t>
+          <t>1099340</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>900</v>
+        <v>820</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>1342227</t>
+          <t>1173613</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -2151,37 +2151,37 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>1315646</t>
+          <t>825327</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>990</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>1338647</t>
+          <t>1254903</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>910</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>1342207</t>
+          <t>1254949</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>1130</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>1342206</t>
+          <t>1340103</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -2191,207 +2191,207 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>1257442</t>
+          <t>1338199</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>1150</v>
+        <v>860</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>1342208</t>
+          <t>1338200</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>1130</v>
+        <v>830</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>1344109</t>
+          <t>1095355</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>870</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>1255617</t>
+          <t>1247617</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>1140</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>1090100</t>
+          <t>1315633</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>1150</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>1340127</t>
+          <t>1340104</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>1100</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>1340095</t>
+          <t>1342229</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>720</v>
+        <v>700</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>1255847</t>
+          <t>1254880</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>1010</v>
+        <v>860</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>1340101</t>
+          <t>1255867</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>1110</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>179426</t>
+          <t>1340657</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>1180</v>
+        <v>900</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>1173624</t>
+          <t>1342227</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>760</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>1340102</t>
+          <t>1315646</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>1110</v>
+        <v>990</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>1102209</t>
+          <t>1338647</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>880</v>
+        <v>910</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>1338648</t>
+          <t>1342207</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>860</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>1342215</t>
+          <t>1342206</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>920</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>1052676</t>
+          <t>1257442</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>760</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>1173618</t>
+          <t>1342208</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>1200</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>1255759</t>
+          <t>1344109</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>1100</v>
+        <v>870</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>1265201</t>
+          <t>1255617</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>1200</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>1340096</t>
+          <t>1090100</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>920</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>1173619</t>
+          <t>1340127</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -2401,447 +2401,447 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>1340113</t>
+          <t>1340095</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>1110</v>
+        <v>720</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>1265205</t>
+          <t>1255847</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>990</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>1315645</t>
+          <t>1340101</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>990</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>1315643</t>
+          <t>179426</t>
         </is>
       </c>
       <c r="B202" t="n">
-        <v>1200</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>1315644</t>
+          <t>1173624</t>
         </is>
       </c>
       <c r="B203" t="n">
-        <v>990</v>
+        <v>760</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>1172331</t>
+          <t>1340102</t>
         </is>
       </c>
       <c r="B204" t="n">
-        <v>910</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>1172332</t>
+          <t>1102209</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>820</v>
+        <v>880</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>1265196</t>
+          <t>1338648</t>
         </is>
       </c>
       <c r="B206" t="n">
-        <v>990</v>
+        <v>860</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>1257448</t>
+          <t>1342215</t>
         </is>
       </c>
       <c r="B207" t="n">
-        <v>990</v>
+        <v>920</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>1340106</t>
+          <t>1052676</t>
         </is>
       </c>
       <c r="B208" t="n">
-        <v>1170</v>
+        <v>760</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>1338611</t>
+          <t>1173618</t>
         </is>
       </c>
       <c r="B209" t="n">
-        <v>940</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>1342223</t>
+          <t>1340109</t>
         </is>
       </c>
       <c r="B210" t="n">
-        <v>760</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>1340118</t>
+          <t>1255759</t>
         </is>
       </c>
       <c r="B211" t="n">
-        <v>1250</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>1342224</t>
+          <t>1265201</t>
         </is>
       </c>
       <c r="B212" t="n">
-        <v>760</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>1340116</t>
+          <t>1340096</t>
         </is>
       </c>
       <c r="B213" t="n">
-        <v>1220</v>
+        <v>920</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>1340117</t>
+          <t>1173619</t>
         </is>
       </c>
       <c r="B214" t="n">
-        <v>1220</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>1052948</t>
+          <t>1340113</t>
         </is>
       </c>
       <c r="B215" t="n">
-        <v>1130</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>1342214</t>
+          <t>1265205</t>
         </is>
       </c>
       <c r="B216" t="n">
-        <v>1140</v>
+        <v>990</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>1344546</t>
+          <t>1315645</t>
         </is>
       </c>
       <c r="B217" t="n">
-        <v>1100</v>
+        <v>990</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>1342205</t>
+          <t>1315643</t>
         </is>
       </c>
       <c r="B218" t="n">
-        <v>1140</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>1340107</t>
+          <t>1315644</t>
         </is>
       </c>
       <c r="B219" t="n">
-        <v>1140</v>
+        <v>990</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>1254765</t>
+          <t>1172331</t>
         </is>
       </c>
       <c r="B220" t="n">
-        <v>1140</v>
+        <v>910</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>1340105</t>
+          <t>1172332</t>
         </is>
       </c>
       <c r="B221" t="n">
-        <v>1140</v>
+        <v>820</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>1257443</t>
+          <t>1265196</t>
         </is>
       </c>
       <c r="B222" t="n">
-        <v>920</v>
+        <v>990</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>1257445</t>
+          <t>1257448</t>
         </is>
       </c>
       <c r="B223" t="n">
-        <v>910</v>
+        <v>990</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>1338610</t>
+          <t>1340106</t>
         </is>
       </c>
       <c r="B224" t="n">
-        <v>910</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>1340108</t>
+          <t>1338611</t>
         </is>
       </c>
       <c r="B225" t="n">
-        <v>1140</v>
+        <v>940</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>1315637</t>
+          <t>1342223</t>
         </is>
       </c>
       <c r="B226" t="n">
-        <v>990</v>
+        <v>760</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>1173628</t>
+          <t>1340118</t>
         </is>
       </c>
       <c r="B227" t="n">
-        <v>920</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>1255758</t>
+          <t>1342224</t>
         </is>
       </c>
       <c r="B228" t="n">
-        <v>1100</v>
+        <v>760</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>1098104</t>
+          <t>1340116</t>
         </is>
       </c>
       <c r="B229" t="n">
-        <v>1120</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>1340111</t>
+          <t>1340117</t>
         </is>
       </c>
       <c r="B230" t="n">
-        <v>1110</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>1342226</t>
+          <t>1052948</t>
         </is>
       </c>
       <c r="B231" t="n">
-        <v>730</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>1340112</t>
+          <t>1342214</t>
         </is>
       </c>
       <c r="B232" t="n">
-        <v>1170</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>1315638</t>
+          <t>1344546</t>
         </is>
       </c>
       <c r="B233" t="n">
-        <v>1090</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>1342213</t>
+          <t>1342205</t>
         </is>
       </c>
       <c r="B234" t="n">
-        <v>700</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>1342222</t>
+          <t>1340107</t>
         </is>
       </c>
       <c r="B235" t="n">
-        <v>950</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>1342218</t>
+          <t>1254765</t>
         </is>
       </c>
       <c r="B236" t="n">
-        <v>940</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>1342217</t>
+          <t>1340105</t>
         </is>
       </c>
       <c r="B237" t="n">
-        <v>980</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>1342211</t>
+          <t>1257443</t>
         </is>
       </c>
       <c r="B238" t="n">
-        <v>970</v>
+        <v>920</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>1098146</t>
+          <t>1257445</t>
         </is>
       </c>
       <c r="B239" t="n">
-        <v>880</v>
+        <v>910</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>947765</t>
+          <t>1338610</t>
         </is>
       </c>
       <c r="B240" t="n">
-        <v>820</v>
+        <v>910</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>1340119</t>
+          <t>1340108</t>
         </is>
       </c>
       <c r="B241" t="n">
-        <v>910</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>1340120</t>
+          <t>1315637</t>
         </is>
       </c>
       <c r="B242" t="n">
-        <v>920</v>
+        <v>990</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>1342209</t>
+          <t>1173628</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -2851,137 +2851,137 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>1172326</t>
+          <t>1255758</t>
         </is>
       </c>
       <c r="B244" t="n">
-        <v>920</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>1099732</t>
+          <t>1098104</t>
         </is>
       </c>
       <c r="B245" t="n">
-        <v>920</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>1342221</t>
+          <t>1340111</t>
         </is>
       </c>
       <c r="B246" t="n">
-        <v>880</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>1342230</t>
+          <t>1342226</t>
         </is>
       </c>
       <c r="B247" t="n">
-        <v>660</v>
+        <v>730</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>1315641</t>
+          <t>1340112</t>
         </is>
       </c>
       <c r="B248" t="n">
-        <v>1200</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>1100670</t>
+          <t>1315638</t>
         </is>
       </c>
       <c r="B249" t="n">
-        <v>650</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>1342228</t>
+          <t>1342213</t>
         </is>
       </c>
       <c r="B250" t="n">
-        <v>660</v>
+        <v>700</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>1340125</t>
+          <t>1342222</t>
         </is>
       </c>
       <c r="B251" t="n">
-        <v>870</v>
+        <v>950</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>1342225</t>
+          <t>1342218</t>
         </is>
       </c>
       <c r="B252" t="n">
-        <v>760</v>
+        <v>940</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>1342204</t>
+          <t>1342217</t>
         </is>
       </c>
       <c r="B253" t="n">
-        <v>660</v>
+        <v>980</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>1344110</t>
+          <t>1342211</t>
         </is>
       </c>
       <c r="B254" t="n">
-        <v>940</v>
+        <v>970</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>1173132</t>
+          <t>1098146</t>
         </is>
       </c>
       <c r="B255" t="n">
-        <v>990</v>
+        <v>880</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>1340650</t>
+          <t>947765</t>
         </is>
       </c>
       <c r="B256" t="n">
-        <v>1070</v>
+        <v>820</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>1338649</t>
+          <t>1340119</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -2991,67 +2991,67 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>1256314</t>
+          <t>1340120</t>
         </is>
       </c>
       <c r="B258" t="n">
-        <v>990</v>
+        <v>920</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>1342212</t>
+          <t>1342209</t>
         </is>
       </c>
       <c r="B259" t="n">
-        <v>700</v>
+        <v>920</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>1340115</t>
+          <t>1172326</t>
         </is>
       </c>
       <c r="B260" t="n">
-        <v>1170</v>
+        <v>920</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>557446</t>
+          <t>1099732</t>
         </is>
       </c>
       <c r="B261" t="n">
-        <v>1160</v>
+        <v>920</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>1340114</t>
+          <t>1342221</t>
         </is>
       </c>
       <c r="B262" t="n">
-        <v>1170</v>
+        <v>880</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>1315648</t>
+          <t>1342230</t>
         </is>
       </c>
       <c r="B263" t="n">
-        <v>990</v>
+        <v>660</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>1315640</t>
+          <t>1315641</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -3061,97 +3061,97 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>1173625</t>
+          <t>1100670</t>
         </is>
       </c>
       <c r="B265" t="n">
-        <v>920</v>
+        <v>650</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>1342216</t>
+          <t>1342228</t>
         </is>
       </c>
       <c r="B266" t="n">
-        <v>980</v>
+        <v>660</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>1053230</t>
+          <t>1340125</t>
         </is>
       </c>
       <c r="B267" t="n">
-        <v>880</v>
+        <v>870</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>1342220</t>
+          <t>1340110</t>
         </is>
       </c>
       <c r="B268" t="n">
-        <v>950</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>1053223</t>
+          <t>1342225</t>
         </is>
       </c>
       <c r="B269" t="n">
-        <v>910</v>
+        <v>760</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>1342482</t>
+          <t>1342204</t>
         </is>
       </c>
       <c r="B270" t="n">
-        <v>950</v>
+        <v>660</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>1340649</t>
+          <t>1344110</t>
         </is>
       </c>
       <c r="B271" t="n">
-        <v>1010</v>
+        <v>940</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>1340651</t>
+          <t>1173132</t>
         </is>
       </c>
       <c r="B272" t="n">
-        <v>970</v>
+        <v>990</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>947769</t>
+          <t>1340650</t>
         </is>
       </c>
       <c r="B273" t="n">
-        <v>820</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>1340122</t>
+          <t>1338649</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -3161,67 +3161,67 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>1340123</t>
+          <t>1256314</t>
         </is>
       </c>
       <c r="B275" t="n">
-        <v>920</v>
+        <v>990</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>1342210</t>
+          <t>1342212</t>
         </is>
       </c>
       <c r="B276" t="n">
-        <v>920</v>
+        <v>700</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>1342219</t>
+          <t>1340115</t>
         </is>
       </c>
       <c r="B277" t="n">
-        <v>880</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>1342231</t>
+          <t>557446</t>
         </is>
       </c>
       <c r="B278" t="n">
-        <v>590</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>1315642</t>
+          <t>1340114</t>
         </is>
       </c>
       <c r="B279" t="n">
-        <v>1200</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>1340124</t>
+          <t>1315648</t>
         </is>
       </c>
       <c r="B280" t="n">
-        <v>650</v>
+        <v>990</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>556749</t>
+          <t>1315640</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -3231,151 +3231,1051 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>557111</t>
+          <t>1315639</t>
         </is>
       </c>
       <c r="B282" t="n">
-        <v>1200</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>182832</t>
+          <t>1173625</t>
         </is>
       </c>
       <c r="B283" t="n">
-        <v>1200</v>
+        <v>920</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>1310892</t>
+          <t>1342216</t>
         </is>
       </c>
       <c r="B284" t="n">
-        <v>1200</v>
+        <v>980</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>1345457</t>
+          <t>1053230</t>
         </is>
       </c>
       <c r="B285" t="n">
-        <v>1100</v>
+        <v>880</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>1222403</t>
+          <t>1342220</t>
         </is>
       </c>
       <c r="B286" t="n">
-        <v>210</v>
+        <v>950</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>110508</t>
+          <t>1053223</t>
         </is>
       </c>
       <c r="B287" t="n">
-        <v>150</v>
+        <v>910</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>142989</t>
+          <t>1342482</t>
         </is>
       </c>
       <c r="B288" t="n">
-        <v>150</v>
+        <v>950</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>143523</t>
+          <t>1340649</t>
         </is>
       </c>
       <c r="B289" t="n">
-        <v>90</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>1140064</t>
+          <t>1340651</t>
         </is>
       </c>
       <c r="B290" t="n">
-        <v>110</v>
+        <v>970</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>1222401</t>
+          <t>947769</t>
         </is>
       </c>
       <c r="B291" t="n">
-        <v>180</v>
+        <v>820</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>154190</t>
+          <t>1340122</t>
         </is>
       </c>
       <c r="B292" t="n">
-        <v>180</v>
+        <v>910</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>1011430</t>
+          <t>1340123</t>
         </is>
       </c>
       <c r="B293" t="n">
-        <v>80</v>
+        <v>920</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>1257898</t>
+          <t>1342210</t>
         </is>
       </c>
       <c r="B294" t="n">
-        <v>110</v>
+        <v>920</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>1326441</t>
+          <t>1342219</t>
         </is>
       </c>
       <c r="B295" t="n">
-        <v>110</v>
+        <v>880</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
+          <t>1342231</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>1315642</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>1340124</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>1261159</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>1880</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>1312849</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>1341376</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>1930</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>1261158</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>1830</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>1134244</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>1312875</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>1260884</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>2170</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>1311775</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>1310984</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>2260</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>1310985</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>2260</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>1187109</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>1285456</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>1213632</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>1223886</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>1140072</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>1177665</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>1135752</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>1342495</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>144506</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>2550</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>166013</t>
+        </is>
+      </c>
+      <c r="B318" t="n">
+        <v>2550</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>1238779</t>
+        </is>
+      </c>
+      <c r="B319" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>1258147</t>
+        </is>
+      </c>
+      <c r="B320" t="n">
+        <v>1930</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>1286229</t>
+        </is>
+      </c>
+      <c r="B321" t="n">
+        <v>1930</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>1342334</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>1013654</t>
+        </is>
+      </c>
+      <c r="B323" t="n">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>556749</t>
+        </is>
+      </c>
+      <c r="B324" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>557111</t>
+        </is>
+      </c>
+      <c r="B325" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>89807</t>
+        </is>
+      </c>
+      <c r="B326" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>182832</t>
+        </is>
+      </c>
+      <c r="B327" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>822861</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>1223985</t>
+        </is>
+      </c>
+      <c r="B329" t="n">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>1310892</t>
+        </is>
+      </c>
+      <c r="B330" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>556757</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>556768</t>
+        </is>
+      </c>
+      <c r="B332" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>556770</t>
+        </is>
+      </c>
+      <c r="B333" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>10102</t>
+        </is>
+      </c>
+      <c r="B334" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>10114</t>
+        </is>
+      </c>
+      <c r="B335" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>72343</t>
+        </is>
+      </c>
+      <c r="B336" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>556764</t>
+        </is>
+      </c>
+      <c r="B337" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>556767</t>
+        </is>
+      </c>
+      <c r="B338" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>556769</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>10103</t>
+        </is>
+      </c>
+      <c r="B340" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>10117</t>
+        </is>
+      </c>
+      <c r="B341" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>42760</t>
+        </is>
+      </c>
+      <c r="B342" t="n">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>1344193</t>
+        </is>
+      </c>
+      <c r="B343" t="n">
+        <v>1830</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>1261176</t>
+        </is>
+      </c>
+      <c r="B344" t="n">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>1310988</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>1880</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>1103158</t>
+        </is>
+      </c>
+      <c r="B346" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>1310991</t>
+        </is>
+      </c>
+      <c r="B347" t="n">
+        <v>1880</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>1345243</t>
+        </is>
+      </c>
+      <c r="B348" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>1172000</t>
+        </is>
+      </c>
+      <c r="B349" t="n">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>1342518</t>
+        </is>
+      </c>
+      <c r="B350" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>151464</t>
+        </is>
+      </c>
+      <c r="B351" t="n">
+        <v>2120</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>157837</t>
+        </is>
+      </c>
+      <c r="B352" t="n">
+        <v>2120</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>1140775</t>
+        </is>
+      </c>
+      <c r="B353" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>1164790</t>
+        </is>
+      </c>
+      <c r="B354" t="n">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>1088235</t>
+        </is>
+      </c>
+      <c r="B355" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>1310891</t>
+        </is>
+      </c>
+      <c r="B356" t="n">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>1091109</t>
+        </is>
+      </c>
+      <c r="B357" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>1170234</t>
+        </is>
+      </c>
+      <c r="B358" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>1015091</t>
+        </is>
+      </c>
+      <c r="B359" t="n">
+        <v>2550</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>993440</t>
+        </is>
+      </c>
+      <c r="B360" t="n">
+        <v>2950</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>1056021</t>
+        </is>
+      </c>
+      <c r="B361" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>18645</t>
+        </is>
+      </c>
+      <c r="B362" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>36003</t>
+        </is>
+      </c>
+      <c r="B363" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>44782</t>
+        </is>
+      </c>
+      <c r="B364" t="n">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>72550</t>
+        </is>
+      </c>
+      <c r="B365" t="n">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>72551</t>
+        </is>
+      </c>
+      <c r="B366" t="n">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>72552</t>
+        </is>
+      </c>
+      <c r="B367" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>18643</t>
+        </is>
+      </c>
+      <c r="B368" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>158305</t>
+        </is>
+      </c>
+      <c r="B369" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>1345457</t>
+        </is>
+      </c>
+      <c r="B370" t="n">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>1222403</t>
+        </is>
+      </c>
+      <c r="B371" t="n">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>110508</t>
+        </is>
+      </c>
+      <c r="B372" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>142989</t>
+        </is>
+      </c>
+      <c r="B373" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>63528</t>
+        </is>
+      </c>
+      <c r="B374" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>96395</t>
+        </is>
+      </c>
+      <c r="B375" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>96388</t>
+        </is>
+      </c>
+      <c r="B376" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>143523</t>
+        </is>
+      </c>
+      <c r="B377" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>1140064</t>
+        </is>
+      </c>
+      <c r="B378" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>1222401</t>
+        </is>
+      </c>
+      <c r="B379" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>96392</t>
+        </is>
+      </c>
+      <c r="B380" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>154190</t>
+        </is>
+      </c>
+      <c r="B381" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>1011430</t>
+        </is>
+      </c>
+      <c r="B382" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>1257898</t>
+        </is>
+      </c>
+      <c r="B383" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>1326441</t>
+        </is>
+      </c>
+      <c r="B384" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
           <t>1222402</t>
         </is>
       </c>
-      <c r="B296" t="n">
+      <c r="B385" t="n">
         <v>140</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>63526</t>
+        </is>
+      </c>
+      <c r="B386" t="n">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>